<commit_message>
Update impedance workflows and add standalone single-file pipeline
</commit_message>
<xml_diff>
--- a/gcv_lambda_s2422_result.xlsx
+++ b/gcv_lambda_s2422_result.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mitra\Downloads\matlab analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2362F926-9A6B-489B-BB96-6F622FE20B3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FB46386-7BDF-4B7B-96B4-A51441FB62A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{8C9ABBA4-03BE-4B52-B0F1-B0A7846E19F5}"/>
   </bookViews>
@@ -17,6 +17,7 @@
     <sheet name="summary" sheetId="2" r:id="rId2"/>
     <sheet name="lambda_scan" sheetId="3" r:id="rId3"/>
     <sheet name="drt_optimal" sheetId="4" r:id="rId4"/>
+    <sheet name="weights" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
   <si>
     <t>method</t>
   </si>
@@ -75,7 +76,61 @@
     <t>gamma_opt</t>
   </si>
   <si>
-    <t>GCV</t>
+    <t>weight_mode</t>
+  </si>
+  <si>
+    <t>w_re</t>
+  </si>
+  <si>
+    <t>w_im</t>
+  </si>
+  <si>
+    <t>sigma_re</t>
+  </si>
+  <si>
+    <t>sigma_im</t>
+  </si>
+  <si>
+    <t>auto_noise</t>
+  </si>
+  <si>
+    <t>GCV_IMAG_INV_REIM_SCORE</t>
+  </si>
+  <si>
+    <t>residual_norm_im</t>
+  </si>
+  <si>
+    <t>solution_norm_im</t>
+  </si>
+  <si>
+    <t>mean_residual_im</t>
+  </si>
+  <si>
+    <t>R_inf_im</t>
+  </si>
+  <si>
+    <t>trace_H_im</t>
+  </si>
+  <si>
+    <t>gcv_score_im</t>
+  </si>
+  <si>
+    <t>residual_norm_re</t>
+  </si>
+  <si>
+    <t>solution_norm_re</t>
+  </si>
+  <si>
+    <t>mean_residual_re</t>
+  </si>
+  <si>
+    <t>R_inf_re</t>
+  </si>
+  <si>
+    <t>trace_H_re</t>
+  </si>
+  <si>
+    <t>gcv_score_re</t>
   </si>
 </sst>
 </file>
@@ -464,25 +519,25 @@
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="B2">
-        <v>5.9948425031894088E-3</v>
+        <v>7.8804628156699122E-4</v>
       </c>
       <c r="C2">
-        <v>0</v>
+        <v>152.0417430958347</v>
       </c>
       <c r="D2">
-        <v>4073.7327609418112</v>
+        <v>665.01295882896079</v>
       </c>
       <c r="E2">
-        <v>21294.090669281271</v>
+        <v>22358.784442777327</v>
       </c>
       <c r="F2">
-        <v>127.18077294705621</v>
+        <v>20.153629755781694</v>
       </c>
       <c r="G2">
-        <v>16852023.22630221</v>
+        <v>1388.01292817065</v>
       </c>
       <c r="H2" t="s">
         <v>7</v>
@@ -498,227 +553,1278 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A24C57CF-79A7-47C3-9A0A-A4E94E547A46}">
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:M31"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>9</v>
       </c>
       <c r="B1" t="s">
-        <v>3</v>
+        <v>19</v>
       </c>
       <c r="C1" t="s">
-        <v>4</v>
+        <v>20</v>
       </c>
       <c r="D1" t="s">
-        <v>5</v>
+        <v>21</v>
       </c>
       <c r="E1" t="s">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="F1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+        <v>23</v>
+      </c>
+      <c r="G1" t="s">
+        <v>24</v>
+      </c>
+      <c r="H1" t="s">
+        <v>25</v>
+      </c>
+      <c r="I1" t="s">
+        <v>26</v>
+      </c>
+      <c r="J1" t="s">
+        <v>27</v>
+      </c>
+      <c r="K1" t="s">
+        <v>28</v>
+      </c>
+      <c r="L1" t="s">
+        <v>29</v>
+      </c>
+      <c r="M1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2">
-        <v>1E-4</v>
+        <v>9.9999999999999995E-7</v>
       </c>
       <c r="B2">
-        <v>4179.7199470204223</v>
+        <v>669.6716513847266</v>
       </c>
       <c r="C2">
-        <v>26325.832018698467</v>
+        <v>39413.108394001232</v>
       </c>
       <c r="D2">
-        <v>130.24598702582696</v>
+        <v>20.00787811438769</v>
       </c>
       <c r="E2">
-        <v>0</v>
+        <v>160.52126592882675</v>
       </c>
       <c r="F2">
-        <v>17649410.673200037</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+        <v>19.506219976360811</v>
+      </c>
+      <c r="G2">
+        <v>1545.5808871351674</v>
+      </c>
+      <c r="H2">
+        <v>810.03064573641018</v>
+      </c>
+      <c r="I2">
+        <v>38128.325738584273</v>
+      </c>
+      <c r="J2">
+        <v>19.956771130770974</v>
+      </c>
+      <c r="K2">
+        <v>3.8182412333871354</v>
+      </c>
+      <c r="L2">
+        <v>19.106633326257377</v>
+      </c>
+      <c r="M2">
+        <v>2250.2848334152072</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A3">
-        <v>2.7825594022071258E-4</v>
+        <v>1.6102620275609392E-6</v>
       </c>
       <c r="B3">
-        <v>4159.3150085840443</v>
+        <v>669.54572266138246</v>
       </c>
       <c r="C3">
-        <v>24611.874946423628</v>
+        <v>36033.506180637502</v>
       </c>
       <c r="D3">
-        <v>129.06207937388879</v>
+        <v>19.992311631416076</v>
       </c>
       <c r="E3">
-        <v>0</v>
+        <v>160.37396417120837</v>
       </c>
       <c r="F3">
-        <v>17480226.020838417</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+        <v>18.950796188834381</v>
+      </c>
+      <c r="G3">
+        <v>1534.4915714574934</v>
+      </c>
+      <c r="H3">
+        <v>809.99656719380584</v>
+      </c>
+      <c r="I3">
+        <v>35421.99662120601</v>
+      </c>
+      <c r="J3">
+        <v>19.965131342779301</v>
+      </c>
+      <c r="K3">
+        <v>3.8295688162178494</v>
+      </c>
+      <c r="L3">
+        <v>18.552077990529956</v>
+      </c>
+      <c r="M3">
+        <v>2234.8528952657866</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A4">
-        <v>7.7426368268112698E-4</v>
+        <v>2.5929437974046672E-6</v>
       </c>
       <c r="B4">
-        <v>4129.1557053182651</v>
+        <v>669.55410512569836</v>
       </c>
       <c r="C4">
-        <v>23435.520000905173</v>
+        <v>33476.617848113608</v>
       </c>
       <c r="D4">
-        <v>127.52863591312641</v>
+        <v>19.984335180448916</v>
       </c>
       <c r="E4">
-        <v>0</v>
+        <v>160.26453253451933</v>
       </c>
       <c r="F4">
-        <v>17235105.133522302</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+        <v>18.395357301472732</v>
+      </c>
+      <c r="G4">
+        <v>1524.1282015601496</v>
+      </c>
+      <c r="H4">
+        <v>809.95284722919791</v>
+      </c>
+      <c r="I4">
+        <v>33238.779294060914</v>
+      </c>
+      <c r="J4">
+        <v>19.974241761061283</v>
+      </c>
+      <c r="K4">
+        <v>3.8432729580834475</v>
+      </c>
+      <c r="L4">
+        <v>17.997615936675878</v>
+      </c>
+      <c r="M4">
+        <v>2219.5275623930802</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A5">
-        <v>2.1544346900318821E-3</v>
+        <v>4.1753189365604001E-6</v>
       </c>
       <c r="B5">
-        <v>4090.3174749054651</v>
+        <v>669.70184498056028</v>
       </c>
       <c r="C5">
-        <v>22323.586804060749</v>
+        <v>31773.253044474837</v>
       </c>
       <c r="D5">
-        <v>126.48390913261967</v>
+        <v>19.98882063818262</v>
       </c>
       <c r="E5">
-        <v>0</v>
+        <v>160.19801929270287</v>
       </c>
       <c r="F5">
-        <v>16932781.208686311</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+        <v>17.83989577797761</v>
+      </c>
+      <c r="G5">
+        <v>1514.4995365931397</v>
+      </c>
+      <c r="H5">
+        <v>809.90520856286037</v>
+      </c>
+      <c r="I5">
+        <v>31373.991649197644</v>
+      </c>
+      <c r="J5">
+        <v>19.987605380828153</v>
+      </c>
+      <c r="K5">
+        <v>3.8612935658473182</v>
+      </c>
+      <c r="L5">
+        <v>17.443253198628273</v>
+      </c>
+      <c r="M5">
+        <v>2204.3390294767096</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A6">
-        <v>5.9948425031894088E-3</v>
+        <v>6.7233575364993352E-6</v>
       </c>
       <c r="B6">
-        <v>4073.7327609418112</v>
+        <v>669.63447926523861</v>
       </c>
       <c r="C6">
-        <v>21294.090669281271</v>
+        <v>29205.413679542919</v>
       </c>
       <c r="D6">
-        <v>127.18077294705621</v>
+        <v>19.975064470759204</v>
       </c>
       <c r="E6">
-        <v>0</v>
+        <v>159.90996564282773</v>
       </c>
       <c r="F6">
-        <v>16852023.22630221</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+        <v>17.284402600388582</v>
+      </c>
+      <c r="G6">
+        <v>1503.9990272287769</v>
+      </c>
+      <c r="H6">
+        <v>809.80183888584304</v>
+      </c>
+      <c r="I6">
+        <v>29556.207725723452</v>
+      </c>
+      <c r="J6">
+        <v>20.006618618093132</v>
+      </c>
+      <c r="K6">
+        <v>3.8898329860412773</v>
+      </c>
+      <c r="L6">
+        <v>16.888996528385448</v>
+      </c>
+      <c r="M6">
+        <v>2189.0056163810204</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A7">
-        <v>1.6681005372000592E-2</v>
+        <v>1.0826367338740541E-5</v>
       </c>
       <c r="B7">
-        <v>4153.9709814107746</v>
+        <v>669.8158761746439</v>
       </c>
       <c r="C7">
-        <v>20461.816664823109</v>
+        <v>27459.284146681628</v>
       </c>
       <c r="D7">
-        <v>132.46213812095769</v>
+        <v>19.973348096447406</v>
       </c>
       <c r="E7">
-        <v>0</v>
+        <v>159.69122038351165</v>
       </c>
       <c r="F7">
-        <v>17685601.640128158</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+        <v>16.728867083018137</v>
+      </c>
+      <c r="G7">
+        <v>1494.7145366998641</v>
+      </c>
+      <c r="H7">
+        <v>809.65482690977694</v>
+      </c>
+      <c r="I7">
+        <v>28242.518508658661</v>
+      </c>
+      <c r="J7">
+        <v>20.027935945928881</v>
+      </c>
+      <c r="K7">
+        <v>3.9258009877219879</v>
+      </c>
+      <c r="L7">
+        <v>16.334853735484792</v>
+      </c>
+      <c r="M7">
+        <v>2173.5964419038773</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A8">
-        <v>4.6415888336127774E-2</v>
+        <v>1.7433288221999873E-5</v>
       </c>
       <c r="B8">
-        <v>4548.8213620263841</v>
+        <v>669.91501552356829</v>
       </c>
       <c r="C8">
-        <v>19764.814925924336</v>
+        <v>25956.211336116899</v>
       </c>
       <c r="D8">
-        <v>151.43981566495444</v>
+        <v>19.961605380001206</v>
       </c>
       <c r="E8">
-        <v>0</v>
+        <v>159.34752605265254</v>
       </c>
       <c r="F8">
-        <v>21755554.038188674</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+        <v>16.173276514545087</v>
+      </c>
+      <c r="G8">
+        <v>1485.1549848275713</v>
+      </c>
+      <c r="H8">
+        <v>809.41674224281098</v>
+      </c>
+      <c r="I8">
+        <v>27286.029062170612</v>
+      </c>
+      <c r="J8">
+        <v>20.050519031420848</v>
+      </c>
+      <c r="K8">
+        <v>3.9717161199237632</v>
+      </c>
+      <c r="L8">
+        <v>15.780834158085622</v>
+      </c>
+      <c r="M8">
+        <v>2157.8614764716563</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A9">
-        <v>0.12915496650148839</v>
+        <v>2.8072162039411757E-5</v>
       </c>
       <c r="B9">
-        <v>6025.2027123393091</v>
+        <v>670.05246485283442</v>
       </c>
       <c r="C9">
-        <v>18856.978700436746</v>
+        <v>24953.300377014002</v>
       </c>
       <c r="D9">
-        <v>213.57965924824146</v>
+        <v>19.957323391824477</v>
       </c>
       <c r="E9">
-        <v>0</v>
+        <v>159.01102169788214</v>
       </c>
       <c r="F9">
-        <v>40894119.661059096</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+        <v>15.617615745362819</v>
+      </c>
+      <c r="G9">
+        <v>1475.857150243346</v>
+      </c>
+      <c r="H9">
+        <v>809.33946536209635</v>
+      </c>
+      <c r="I9">
+        <v>25986.050078802116</v>
+      </c>
+      <c r="J9">
+        <v>20.105530093970426</v>
+      </c>
+      <c r="K9">
+        <v>4.0458966202974178</v>
+      </c>
+      <c r="L9">
+        <v>15.22694920943705</v>
+      </c>
+      <c r="M9">
+        <v>2143.142663308593</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A10">
-        <v>0.35938136638046259</v>
+        <v>4.5203536563602408E-5</v>
       </c>
       <c r="B10">
-        <v>10774.578921007269</v>
+        <v>669.68234478007378</v>
       </c>
       <c r="C10">
-        <v>17222.210756096585</v>
+        <v>24248.908210713336</v>
       </c>
       <c r="D10">
-        <v>390.00920849524795</v>
+        <v>19.924451049845224</v>
       </c>
       <c r="E10">
-        <v>0</v>
+        <v>158.52720711760915</v>
       </c>
       <c r="F10">
-        <v>156379919.01924053</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+        <v>15.061866494631666</v>
+      </c>
+      <c r="G10">
+        <v>1464.4278666155399</v>
+      </c>
+      <c r="H10">
+        <v>809.52595763208365</v>
+      </c>
+      <c r="I10">
+        <v>24786.150580631267</v>
+      </c>
+      <c r="J10">
+        <v>20.17970365080939</v>
+      </c>
+      <c r="K10">
+        <v>4.1255755292303142</v>
+      </c>
+      <c r="L10">
+        <v>14.673213195664866</v>
+      </c>
+      <c r="M10">
+        <v>2129.962747429046</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A11">
+        <v>7.2789538439831455E-5</v>
+      </c>
+      <c r="B11">
+        <v>668.98193850884775</v>
+      </c>
+      <c r="C11">
+        <v>23735.944326723235</v>
+      </c>
+      <c r="D11">
+        <v>19.885463895359823</v>
+      </c>
+      <c r="E11">
+        <v>157.92218595801532</v>
+      </c>
+      <c r="F11">
+        <v>14.506006457950948</v>
+      </c>
+      <c r="G11">
+        <v>1451.6827041781564</v>
+      </c>
+      <c r="H11">
+        <v>809.51773793750442</v>
+      </c>
+      <c r="I11">
+        <v>24044.60636473247</v>
+      </c>
+      <c r="J11">
+        <v>20.24829789254122</v>
+      </c>
+      <c r="K11">
+        <v>4.2157084168367032</v>
+      </c>
+      <c r="L11">
+        <v>14.119644300521569</v>
+      </c>
+      <c r="M11">
+        <v>2115.8962534803482</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A12">
+        <v>1.1721022975334806E-4</v>
+      </c>
+      <c r="B12">
+        <v>668.14418568925089</v>
+      </c>
+      <c r="C12">
+        <v>23384.150365232563</v>
+      </c>
+      <c r="D12">
+        <v>19.839857934690347</v>
+      </c>
+      <c r="E12">
+        <v>157.22784439025682</v>
+      </c>
+      <c r="F12">
+        <v>13.950007969126546</v>
+      </c>
+      <c r="G12">
+        <v>1438.483175684154</v>
+      </c>
+      <c r="H12">
+        <v>809.42372204808669</v>
+      </c>
+      <c r="I12">
+        <v>23569.499684959046</v>
+      </c>
+      <c r="J12">
+        <v>20.324339583595386</v>
+      </c>
+      <c r="K12">
+        <v>4.3164509410754963</v>
+      </c>
+      <c r="L12">
+        <v>13.566266044804678</v>
+      </c>
+      <c r="M12">
+        <v>2101.5275890564967</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A13">
+        <v>1.8873918221350977E-4</v>
+      </c>
+      <c r="B13">
+        <v>666.99099785523833</v>
+      </c>
+      <c r="C13">
+        <v>23096.300936608284</v>
+      </c>
+      <c r="D13">
+        <v>19.777352700861073</v>
+      </c>
+      <c r="E13">
+        <v>156.3275792072007</v>
+      </c>
+      <c r="F13">
+        <v>13.393836152273973</v>
+      </c>
+      <c r="G13">
+        <v>1424.0801812228756</v>
+      </c>
+      <c r="H13">
+        <v>809.54421005329812</v>
+      </c>
+      <c r="I13">
+        <v>23148.760676798858</v>
+      </c>
+      <c r="J13">
+        <v>20.442957522503065</v>
+      </c>
+      <c r="K13">
+        <v>4.4429415825825691</v>
+      </c>
+      <c r="L13">
+        <v>13.013109200988701</v>
+      </c>
+      <c r="M13">
+        <v>2088.4135556975884</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A14">
+        <v>3.039195382313198E-4</v>
+      </c>
+      <c r="B14">
+        <v>665.7363435382274</v>
+      </c>
+      <c r="C14">
+        <v>22860.83317925498</v>
+      </c>
+      <c r="D14">
+        <v>19.763730648295681</v>
+      </c>
+      <c r="E14">
+        <v>155.23419230373202</v>
+      </c>
+      <c r="F14">
+        <v>12.837446310169373</v>
+      </c>
+      <c r="G14">
+        <v>1409.4103608447865</v>
+      </c>
+      <c r="H14">
+        <v>810.2438185743033</v>
+      </c>
+      <c r="I14">
+        <v>22742.473793806432</v>
+      </c>
+      <c r="J14">
+        <v>20.679308649857184</v>
+      </c>
+      <c r="K14">
+        <v>4.5962825173192359</v>
+      </c>
+      <c r="L14">
+        <v>12.460214536605296</v>
+      </c>
+      <c r="M14">
+        <v>2078.4021676988018</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A15">
+        <v>4.8939009184774938E-4</v>
+      </c>
+      <c r="B15">
+        <v>664.70348684200962</v>
+      </c>
+      <c r="C15">
+        <v>22620.828215175185</v>
+      </c>
+      <c r="D15">
+        <v>19.855032147278159</v>
+      </c>
+      <c r="E15">
+        <v>153.82608937406658</v>
+      </c>
+      <c r="F15">
+        <v>12.280780231377925</v>
+      </c>
+      <c r="G15">
+        <v>1395.8387579489804</v>
+      </c>
+      <c r="H15">
+        <v>812.05531609732202</v>
+      </c>
+      <c r="I15">
+        <v>22350.886786739437</v>
+      </c>
+      <c r="J15">
+        <v>21.144926377769362</v>
+      </c>
+      <c r="K15">
+        <v>4.7815853617718229</v>
+      </c>
+      <c r="L15">
+        <v>11.907636604683448</v>
+      </c>
+      <c r="M15">
+        <v>2074.1635055845923</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A16">
+        <v>7.8804628156699122E-4</v>
+      </c>
+      <c r="B16">
+        <v>665.01295882896079</v>
+      </c>
+      <c r="C16">
+        <v>22358.784442777327</v>
+      </c>
+      <c r="D16">
+        <v>20.153629755781694</v>
+      </c>
+      <c r="E16">
+        <v>152.0417430958347</v>
+      </c>
+      <c r="F16">
+        <v>11.723761087500812</v>
+      </c>
+      <c r="G16">
+        <v>1388.01292817065</v>
+      </c>
+      <c r="H16">
+        <v>816.21335774071281</v>
+      </c>
+      <c r="I16">
+        <v>21944.365573863153</v>
+      </c>
+      <c r="J16">
+        <v>21.959841082084726</v>
+      </c>
+      <c r="K16">
+        <v>4.9963682304205692</v>
+      </c>
+      <c r="L16">
+        <v>11.355449058284616</v>
+      </c>
+      <c r="M16">
+        <v>2081.9195265467811</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A17">
+        <v>1.2689610031679222E-3</v>
+      </c>
+      <c r="B17">
+        <v>668.76958923333893</v>
+      </c>
+      <c r="C17">
+        <v>22069.160438005089</v>
+      </c>
+      <c r="D17">
+        <v>20.763526868116177</v>
+      </c>
+      <c r="E17">
+        <v>150.01157045217818</v>
+      </c>
+      <c r="F17">
+        <v>11.166286264144379</v>
+      </c>
+      <c r="G17">
+        <v>1394.5922930970441</v>
+      </c>
+      <c r="H17">
+        <v>824.41493992904657</v>
+      </c>
+      <c r="I17">
+        <v>21530.505692066949</v>
+      </c>
+      <c r="J17">
+        <v>23.218475024006775</v>
+      </c>
+      <c r="K17">
+        <v>5.2270876047323833</v>
+      </c>
+      <c r="L17">
+        <v>10.80375209970693</v>
+      </c>
+      <c r="M17">
+        <v>2110.3020219589339</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A18">
+        <v>2.0433597178569417E-3</v>
+      </c>
+      <c r="B18">
+        <v>679.68635575722965</v>
+      </c>
+      <c r="C18">
+        <v>21731.259014121795</v>
+      </c>
+      <c r="D18">
+        <v>21.895039384920761</v>
+      </c>
+      <c r="E18">
+        <v>147.48335968498341</v>
+      </c>
+      <c r="F18">
+        <v>10.608217601342599</v>
+      </c>
+      <c r="G18">
+        <v>1431.1280879494038</v>
+      </c>
+      <c r="H18">
+        <v>838.64538832446499</v>
+      </c>
+      <c r="I18">
+        <v>21133.952287041244</v>
+      </c>
+      <c r="J18">
+        <v>24.944254965804085</v>
+      </c>
+      <c r="K18">
+        <v>5.4281623158994385</v>
+      </c>
+      <c r="L18">
+        <v>10.252682764880829</v>
+      </c>
+      <c r="M18">
+        <v>2169.7924554272536</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A19">
+        <v>3.2903445623126675E-3</v>
+      </c>
+      <c r="B19">
+        <v>702.82477168474884</v>
+      </c>
+      <c r="C19">
+        <v>21377.657328803518</v>
+      </c>
+      <c r="D19">
+        <v>23.833995179878801</v>
+      </c>
+      <c r="E19">
+        <v>144.95978990072592</v>
+      </c>
+      <c r="F19">
+        <v>10.049368076321192</v>
+      </c>
+      <c r="G19">
+        <v>1520.2953259196961</v>
+      </c>
+      <c r="H19">
+        <v>859.59348699499265</v>
+      </c>
+      <c r="I19">
+        <v>20807.121962095127</v>
+      </c>
+      <c r="J19">
+        <v>26.941223414024623</v>
+      </c>
+      <c r="K19">
+        <v>5.5073588070913431</v>
+      </c>
+      <c r="L19">
+        <v>9.7024291906022633</v>
+      </c>
+      <c r="M19">
+        <v>2265.0057867646806</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A20">
+        <v>5.2983169062837069E-3</v>
+      </c>
+      <c r="B20">
+        <v>743.97371545092506</v>
+      </c>
+      <c r="C20">
+        <v>21025.945981724315</v>
+      </c>
+      <c r="D20">
+        <v>26.630027162201689</v>
+      </c>
+      <c r="E20">
+        <v>142.86464063306971</v>
+      </c>
+      <c r="F20">
+        <v>9.4894842488975719</v>
+      </c>
+      <c r="G20">
+        <v>1692.4873431596495</v>
+      </c>
+      <c r="H20">
+        <v>888.27593098099385</v>
+      </c>
+      <c r="I20">
+        <v>20549.636598656252</v>
+      </c>
+      <c r="J20">
+        <v>29.177146987669907</v>
+      </c>
+      <c r="K20">
+        <v>5.4031439466354634</v>
+      </c>
+      <c r="L20">
+        <v>9.153249950887556</v>
+      </c>
+      <c r="M20">
+        <v>2403.3374008302935</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A21">
+        <v>8.531678524172805E-3</v>
+      </c>
+      <c r="B21">
+        <v>809.34817966459741</v>
+      </c>
+      <c r="C21">
+        <v>20693.140867812519</v>
+      </c>
+      <c r="D21">
+        <v>30.357774244108811</v>
+      </c>
+      <c r="E21">
+        <v>141.89198811003124</v>
+      </c>
+      <c r="F21">
+        <v>8.9282237149124661</v>
+      </c>
+      <c r="G21">
+        <v>1990.030253677786</v>
+      </c>
+      <c r="H21">
+        <v>926.48623810151639</v>
+      </c>
+      <c r="I21">
+        <v>20343.802577157963</v>
+      </c>
+      <c r="J21">
+        <v>31.662483693281786</v>
+      </c>
+      <c r="K21">
+        <v>5.0711603406368697</v>
+      </c>
+      <c r="L21">
+        <v>8.6055001313689274</v>
+      </c>
+      <c r="M21">
+        <v>2598.0571675465881</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A22">
+        <v>1.3738237958832639E-2</v>
+      </c>
+      <c r="B22">
+        <v>907.03344856818808</v>
+      </c>
+      <c r="C22">
+        <v>20387.617189742672</v>
+      </c>
+      <c r="D22">
+        <v>35.231628761818577</v>
+      </c>
+      <c r="E22">
+        <v>143.150407575081</v>
+      </c>
+      <c r="F22">
+        <v>8.3651278138178888</v>
+      </c>
+      <c r="G22">
+        <v>2483.2136936061365</v>
+      </c>
+      <c r="H22">
+        <v>977.71243926990621</v>
+      </c>
+      <c r="I22">
+        <v>20168.995897271347</v>
+      </c>
+      <c r="J22">
+        <v>34.576490484009383</v>
+      </c>
+      <c r="K22">
+        <v>4.4990628071284879</v>
+      </c>
+      <c r="L22">
+        <v>8.0596655278953104</v>
+      </c>
+      <c r="M22">
+        <v>2875.1669790396913</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A23">
+        <v>2.2122162910704502E-2</v>
+      </c>
+      <c r="B23">
+        <v>1051.6512666108704</v>
+      </c>
+      <c r="C23">
+        <v>20103.333636257888</v>
+      </c>
+      <c r="D23">
+        <v>41.925959911213397</v>
+      </c>
+      <c r="E23">
+        <v>148.20512032566128</v>
+      </c>
+      <c r="F23">
+        <v>7.7995916899605398</v>
+      </c>
+      <c r="G23">
+        <v>3316.5500342140208</v>
+      </c>
+      <c r="H23">
+        <v>1046.4678258371484</v>
+      </c>
+      <c r="I23">
+        <v>20008.396260112822</v>
+      </c>
+      <c r="J23">
+        <v>37.968993404053727</v>
+      </c>
+      <c r="K23">
+        <v>3.7198476608083886</v>
+      </c>
+      <c r="L23">
+        <v>7.5164065437645586</v>
+      </c>
+      <c r="M23">
+        <v>3273.2860462884773</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A24">
+        <v>3.562247890262444E-2</v>
+      </c>
+      <c r="B24">
+        <v>1271.8328940905137</v>
+      </c>
+      <c r="C24">
+        <v>19821.875006601287</v>
+      </c>
+      <c r="D24">
+        <v>51.406268973711903</v>
+      </c>
+      <c r="E24">
+        <v>159.68056713649219</v>
+      </c>
+      <c r="F24">
+        <v>7.2308381581208447</v>
+      </c>
+      <c r="G24">
+        <v>4819.1660622189338</v>
+      </c>
+      <c r="H24">
+        <v>1140.0362433058017</v>
+      </c>
+      <c r="I24">
+        <v>19850.717561218833</v>
+      </c>
+      <c r="J24">
+        <v>42.056133616238832</v>
+      </c>
+      <c r="K24">
+        <v>2.8259395870126363</v>
+      </c>
+      <c r="L24">
+        <v>6.9766123943413989</v>
+      </c>
+      <c r="M24">
+        <v>3860.8820863050614</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A25">
+        <v>5.7361525104486812E-2</v>
+      </c>
+      <c r="B25">
+        <v>1620.3631808933437</v>
+      </c>
+      <c r="C25">
+        <v>19511.637149502698</v>
+      </c>
+      <c r="D25">
+        <v>66.168101818382937</v>
+      </c>
+      <c r="E25">
+        <v>181.71116560795309</v>
+      </c>
+      <c r="F25">
+        <v>6.6579106340091236</v>
+      </c>
+      <c r="G25">
+        <v>7771.301712112082</v>
+      </c>
+      <c r="H25">
+        <v>1273.1052213133362</v>
+      </c>
+      <c r="I25">
+        <v>19682.490922749796</v>
+      </c>
+      <c r="J25">
+        <v>47.39236529511944</v>
+      </c>
+      <c r="K25">
+        <v>1.9974886049460021</v>
+      </c>
+      <c r="L25">
+        <v>6.4414649243143582</v>
+      </c>
+      <c r="M25">
+        <v>4785.4864883335385</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A26">
+        <v>9.2367085718738653E-2</v>
+      </c>
+      <c r="B26">
+        <v>2180.5176706353377</v>
+      </c>
+      <c r="C26">
+        <v>19132.635672242963</v>
+      </c>
+      <c r="D26">
+        <v>90.782626241157175</v>
+      </c>
+      <c r="E26">
+        <v>221.51438771564131</v>
+      </c>
+      <c r="F26">
+        <v>6.0797165542096536</v>
+      </c>
+      <c r="G26">
+        <v>13980.695636573826</v>
+      </c>
+      <c r="H26">
+        <v>1471.0816469251051</v>
+      </c>
+      <c r="I26">
+        <v>19489.938797287243</v>
+      </c>
+      <c r="J26">
+        <v>55.032313309571968</v>
+      </c>
+      <c r="K26">
+        <v>1.5761973907837785</v>
+      </c>
+      <c r="L26">
+        <v>5.9125086005902343</v>
+      </c>
+      <c r="M26">
+        <v>6351.2313716803992</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A27">
+        <v>0.14873521072935117</v>
+      </c>
+      <c r="B27">
+        <v>3064.9679778243662</v>
+      </c>
+      <c r="C27">
+        <v>18652.710757993103</v>
+      </c>
+      <c r="D27">
+        <v>128.43161265350506</v>
+      </c>
+      <c r="E27">
+        <v>295.16928644140819</v>
+      </c>
+      <c r="F27">
+        <v>5.4951811038633114</v>
+      </c>
+      <c r="G27">
+        <v>27439.749442883542</v>
+      </c>
+      <c r="H27">
+        <v>1771.8189800737862</v>
+      </c>
+      <c r="I27">
+        <v>19259.544787364419</v>
+      </c>
+      <c r="J27">
+        <v>68.336603888834603</v>
+      </c>
+      <c r="K27">
+        <v>2.2218427062162629</v>
+      </c>
+      <c r="L27">
+        <v>5.3917190643118422</v>
+      </c>
+      <c r="M27">
+        <v>9159.2089155651393</v>
+      </c>
+    </row>
+    <row r="28" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A28">
+        <v>0.23950266199874859</v>
+      </c>
+      <c r="B28">
+        <v>4436.3469632671595</v>
+      </c>
+      <c r="C28">
+        <v>18019.542427815843</v>
+      </c>
+      <c r="D28">
+        <v>185.17682801364364</v>
+      </c>
+      <c r="E28">
+        <v>424.04348659206624</v>
+      </c>
+      <c r="F28">
+        <v>4.9036131522435706</v>
+      </c>
+      <c r="G28">
+        <v>57104.850665407292</v>
+      </c>
+      <c r="H28">
+        <v>2215.3356433342419</v>
+      </c>
+      <c r="I28">
+        <v>18984.577277352579</v>
+      </c>
+      <c r="J28">
+        <v>88.265030898777269</v>
+      </c>
+      <c r="K28">
+        <v>5.1903409224336636</v>
+      </c>
+      <c r="L28">
+        <v>4.8815574324229534</v>
+      </c>
+      <c r="M28">
+        <v>14236.161069643205</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A29">
+        <v>0.38566204211634725</v>
+      </c>
+      <c r="B29">
+        <v>6507.9080892229613</v>
+      </c>
+      <c r="C29">
+        <v>17167.587310197781</v>
+      </c>
+      <c r="D29">
+        <v>269.62326097432481</v>
+      </c>
+      <c r="E29">
+        <v>635.50155707600106</v>
+      </c>
+      <c r="F29">
+        <v>4.3054328140410902</v>
+      </c>
+      <c r="G29">
+        <v>122060.71624336457</v>
+      </c>
+      <c r="H29">
+        <v>2829.5589484837192</v>
+      </c>
+      <c r="I29">
+        <v>18667.860059160368</v>
+      </c>
+      <c r="J29">
+        <v>114.94554818306068</v>
+      </c>
+      <c r="K29">
+        <v>12.750602734151569</v>
+      </c>
+      <c r="L29">
+        <v>4.3849914163507613</v>
+      </c>
+      <c r="M29">
+        <v>23095.084848741073</v>
+      </c>
+    </row>
+    <row r="30" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A30">
+        <v>0.62101694189156165</v>
+      </c>
+      <c r="B30">
+        <v>9526.620182461631</v>
+      </c>
+      <c r="C30">
+        <v>16027.361491817303</v>
+      </c>
+      <c r="D30">
+        <v>391.44125070545402</v>
+      </c>
+      <c r="E30">
+        <v>961.07865589729079</v>
+      </c>
+      <c r="F30">
+        <v>3.7034158603094247</v>
+      </c>
+      <c r="G30">
+        <v>259796.35156456387</v>
+      </c>
+      <c r="H30">
+        <v>3624.3051375186164</v>
+      </c>
+      <c r="I30">
+        <v>18318.600354012015</v>
+      </c>
+      <c r="J30">
+        <v>149.24829462673668</v>
+      </c>
+      <c r="K30">
+        <v>28.716403955060262</v>
+      </c>
+      <c r="L30">
+        <v>3.9054606939670147</v>
+      </c>
+      <c r="M30">
+        <v>37686.837477796551</v>
+      </c>
+    </row>
+    <row r="31" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A31">
         <v>1</v>
       </c>
-      <c r="B11">
-        <v>22643.810080039544</v>
-      </c>
-      <c r="C11">
-        <v>14341.295448627974</v>
-      </c>
-      <c r="D11">
-        <v>792.4311437603933</v>
-      </c>
-      <c r="E11">
-        <v>0</v>
-      </c>
-      <c r="F11">
-        <v>1064831339.3543602</v>
+      <c r="B31">
+        <v>13715.241315404981</v>
+      </c>
+      <c r="C31">
+        <v>14542.88519241392</v>
+      </c>
+      <c r="D31">
+        <v>560.99706507688211</v>
+      </c>
+      <c r="E31">
+        <v>1427.7294056648855</v>
+      </c>
+      <c r="F31">
+        <v>3.1044536475427154</v>
+      </c>
+      <c r="G31">
+        <v>534871.23345524142</v>
+      </c>
+      <c r="H31">
+        <v>4600.0272527145271</v>
+      </c>
+      <c r="I31">
+        <v>17942.718536509059</v>
+      </c>
+      <c r="J31">
+        <v>192.51910826859344</v>
+      </c>
+      <c r="K31">
+        <v>59.032115029023494</v>
+      </c>
+      <c r="L31">
+        <v>3.4467643871451954</v>
+      </c>
+      <c r="M31">
+        <v>60398.5833680656</v>
       </c>
     </row>
   </sheetData>
@@ -1632,7 +2738,7 @@
         <v>4.3256716491808872E-6</v>
       </c>
       <c r="B113">
-        <v>253.4704262883603</v>
+        <v>0</v>
       </c>
     </row>
     <row r="114" spans="1:2" x14ac:dyDescent="0.3">
@@ -1640,7 +2746,7 @@
         <v>4.0496315749164258E-6</v>
       </c>
       <c r="B114">
-        <v>517.63511324693434</v>
+        <v>0</v>
       </c>
     </row>
     <row r="115" spans="1:2" x14ac:dyDescent="0.3">
@@ -1648,7 +2754,7 @@
         <v>3.7912067576309363E-6</v>
       </c>
       <c r="B115">
-        <v>775.76240871300956</v>
+        <v>6.4560464349726159</v>
       </c>
     </row>
     <row r="116" spans="1:2" x14ac:dyDescent="0.3">
@@ -1656,7 +2762,7 @@
         <v>3.549273188559197E-6</v>
       </c>
       <c r="B116">
-        <v>1025.2308656733464</v>
+        <v>447.26530287928324</v>
       </c>
     </row>
     <row r="117" spans="1:2" x14ac:dyDescent="0.3">
@@ -1664,7 +2770,7 @@
         <v>3.3227785017144782E-6</v>
       </c>
       <c r="B117">
-        <v>1263.4700035086446</v>
+        <v>867.87747244553975</v>
       </c>
     </row>
     <row r="118" spans="1:2" x14ac:dyDescent="0.3">
@@ -1672,7 +2778,7 @@
         <v>3.1107373864717825E-6</v>
       </c>
       <c r="B118">
-        <v>1488.0166938573302</v>
+        <v>1263.3952946675824</v>
       </c>
     </row>
     <row r="119" spans="1:2" x14ac:dyDescent="0.3">
@@ -1680,7 +2786,7 @@
         <v>2.9122275668168558E-6</v>
       </c>
       <c r="B119">
-        <v>1696.5735484764161</v>
+        <v>1629.2621191750252</v>
       </c>
     </row>
     <row r="120" spans="1:2" x14ac:dyDescent="0.3">
@@ -1688,7 +2794,7 @@
         <v>2.7263855508468277E-6</v>
       </c>
       <c r="B120">
-        <v>1887.068271640768</v>
+        <v>1961.3856583199311</v>
       </c>
     </row>
     <row r="121" spans="1:2" x14ac:dyDescent="0.3">
@@ -1696,7 +2802,7 @@
         <v>2.5524029103368681E-6</v>
       </c>
       <c r="B121">
-        <v>2057.7084972542521</v>
+        <v>2256.2511722506079</v>
       </c>
     </row>
     <row r="122" spans="1:2" x14ac:dyDescent="0.3">
@@ -1704,7 +2810,7 @@
         <v>2.3895228419262004E-6</v>
       </c>
       <c r="B122">
-        <v>2207.0333196084393</v>
+        <v>2511.0227884432261</v>
       </c>
     </row>
     <row r="123" spans="1:2" x14ac:dyDescent="0.3">
@@ -1712,7 +2818,7 @@
         <v>2.2370368980838674E-6</v>
       </c>
       <c r="B123">
-        <v>2333.9611190096707</v>
+        <v>2723.6316003559905</v>
       </c>
     </row>
     <row r="124" spans="1:2" x14ac:dyDescent="0.3">
@@ -1720,7 +2826,7 @@
         <v>2.094281742188481E-6</v>
       </c>
       <c r="B124">
-        <v>2437.8279460842159</v>
+        <v>2892.8429807577113</v>
       </c>
     </row>
     <row r="125" spans="1:2" x14ac:dyDescent="0.3">
@@ -1728,7 +2834,7 @@
         <v>1.9606364363521399E-6</v>
       </c>
       <c r="B125">
-        <v>2518.4173401005291</v>
+        <v>3018.3028170183952</v>
       </c>
     </row>
     <row r="126" spans="1:2" x14ac:dyDescent="0.3">
@@ -1736,7 +2842,7 @@
         <v>1.8355196127384421E-6</v>
       </c>
       <c r="B126">
-        <v>2575.9810707558031</v>
+        <v>3100.5622230983754</v>
       </c>
     </row>
     <row r="127" spans="1:2" x14ac:dyDescent="0.3">
@@ -1744,7 +2850,7 @@
         <v>1.7183870316856014E-6</v>
       </c>
       <c r="B127">
-        <v>2611.2467584081878</v>
+        <v>3141.0757943833814</v>
       </c>
     </row>
     <row r="128" spans="1:2" x14ac:dyDescent="0.3">
@@ -1752,7 +2858,7 @@
         <v>1.6087292110365337E-6</v>
       </c>
       <c r="B128">
-        <v>2625.4164371797333</v>
+        <v>3142.1787963653705</v>
       </c>
     </row>
     <row r="129" spans="1:2" x14ac:dyDescent="0.3">
@@ -1760,7 +2866,7 @@
         <v>1.5060691337589852E-6</v>
       </c>
       <c r="B129">
-        <v>2620.1503526931888</v>
+        <v>3107.0370840446567</v>
       </c>
     </row>
     <row r="130" spans="1:2" x14ac:dyDescent="0.3">
@@ -1768,7 +2874,7 @@
         <v>1.4099602424104423E-6</v>
       </c>
       <c r="B130">
-        <v>2597.5380971929767</v>
+        <v>3039.5733803624157</v>
       </c>
     </row>
     <row r="131" spans="1:2" x14ac:dyDescent="0.3">
@@ -1776,7 +2882,7 @@
         <v>1.31998448257266E-6</v>
       </c>
       <c r="B131">
-        <v>2560.059251865232</v>
+        <v>2944.3739024972961</v>
       </c>
     </row>
     <row r="132" spans="1:2" x14ac:dyDescent="0.3">
@@ -1784,7 +2890,7 @@
         <v>1.2357504738635233E-6</v>
       </c>
       <c r="B132">
-        <v>2510.5314975479805</v>
+        <v>2826.5745983630604</v>
       </c>
     </row>
     <row r="133" spans="1:2" x14ac:dyDescent="0.3">
@@ -1792,7 +2898,7 @@
         <v>1.1568918058077187E-6</v>
       </c>
       <c r="B133">
-        <v>2452.048008681536</v>
+        <v>2691.7312902470617</v>
       </c>
     </row>
     <row r="134" spans="1:2" x14ac:dyDescent="0.3">
@@ -1800,7 +2906,7 @@
         <v>1.0830654585309727E-6</v>
       </c>
       <c r="B134">
-        <v>2387.9064858268371</v>
+        <v>2545.678855166886</v>
       </c>
     </row>
     <row r="135" spans="1:2" x14ac:dyDescent="0.3">
@@ -1808,7 +2914,7 @@
         <v>1.0139502937306228E-6</v>
       </c>
       <c r="B135">
-        <v>2321.5307575534416</v>
+        <v>2394.3830216821093</v>
       </c>
     </row>
     <row r="136" spans="1:2" x14ac:dyDescent="0.3">
@@ -1816,7 +2922,7 @@
         <v>9.4924567040157453E-7</v>
       </c>
       <c r="B136">
-        <v>2256.387053704444</v>
+        <v>2243.7898689665631</v>
       </c>
     </row>
     <row r="137" spans="1:2" x14ac:dyDescent="0.3">
@@ -1824,7 +2930,7 @@
         <v>8.886701326418348E-7</v>
       </c>
       <c r="B137">
-        <v>2195.8976869900002</v>
+        <v>2099.6784788910854</v>
       </c>
     </row>
     <row r="138" spans="1:2" x14ac:dyDescent="0.3">
@@ -1832,7 +2938,7 @@
         <v>8.3196018735911818E-7</v>
       </c>
       <c r="B138">
-        <v>2143.3539949132228</v>
+        <v>1967.5209392770055</v>
       </c>
     </row>
     <row r="139" spans="1:2" x14ac:dyDescent="0.3">
@@ -1840,7 +2946,7 @@
         <v>7.7886915407006009E-7</v>
       </c>
       <c r="B139">
-        <v>2101.8310318064191</v>
+        <v>1852.354033724079</v>
       </c>
     </row>
     <row r="140" spans="1:2" x14ac:dyDescent="0.3">
@@ -1848,7 +2954,7 @@
         <v>7.2916609287481189E-7</v>
       </c>
       <c r="B140">
-        <v>2074.1061899765937</v>
+        <v>1758.6660261695713</v>
       </c>
     </row>
     <row r="141" spans="1:2" x14ac:dyDescent="0.3">
@@ -1856,7 +2962,7 @@
         <v>6.8263479984152444E-7</v>
       </c>
       <c r="B141">
-        <v>2062.5838639603844</v>
+        <v>1690.3011750176543</v>
       </c>
     </row>
     <row r="142" spans="1:2" x14ac:dyDescent="0.3">
@@ -1864,7 +2970,7 @@
         <v>6.3907287404493479E-7</v>
       </c>
       <c r="B142">
-        <v>2069.2285742088934</v>
+        <v>1650.384135240944</v>
       </c>
     </row>
     <row r="143" spans="1:2" x14ac:dyDescent="0.3">
@@ -1872,7 +2978,7 @@
         <v>5.9829082582498989E-7</v>
       </c>
       <c r="B143">
-        <v>2095.5075574725711</v>
+        <v>1641.2645027359797</v>
       </c>
     </row>
     <row r="144" spans="1:2" x14ac:dyDescent="0.3">
@@ -1880,7 +2986,7 @@
         <v>5.6011126047966451E-7</v>
       </c>
       <c r="B144">
-        <v>2142.3443797057139</v>
+        <v>1664.481773757019</v>
       </c>
     </row>
     <row r="145" spans="1:2" x14ac:dyDescent="0.3">
@@ -1888,7 +2994,7 @@
         <v>5.2436810019201572E-7</v>
       </c>
       <c r="B145">
-        <v>2210.0847399171412</v>
+        <v>1720.7500194836443</v>
       </c>
     </row>
     <row r="146" spans="1:2" x14ac:dyDescent="0.3">
@@ -1896,7 +3002,7 @@
         <v>4.909058682761205E-7</v>
       </c>
       <c r="B146">
-        <v>2298.4749709136008</v>
+        <v>1809.9606207170682</v>
       </c>
     </row>
     <row r="147" spans="1:2" x14ac:dyDescent="0.3">
@@ -1904,7 +3010,7 @@
         <v>4.595790078981068E-7</v>
       </c>
       <c r="B147">
-        <v>2406.6536798558313</v>
+        <v>1931.2008816964635</v>
       </c>
     </row>
     <row r="148" spans="1:2" x14ac:dyDescent="0.3">
@@ -1912,7 +3018,7 @@
         <v>4.3025125163310383E-7</v>
       </c>
       <c r="B148">
-        <v>2533.1558790221452</v>
+        <v>2082.7850698894213</v>
       </c>
     </row>
     <row r="149" spans="1:2" x14ac:dyDescent="0.3">
@@ -1920,7 +3026,7 @@
         <v>4.0279502948780654E-7</v>
       </c>
       <c r="B149">
-        <v>2675.9298337918872</v>
+        <v>2262.2947410805218</v>
       </c>
     </row>
     <row r="150" spans="1:2" x14ac:dyDescent="0.3">
@@ -1928,7 +3034,7 @@
         <v>3.7709090910530791E-7</v>
       </c>
       <c r="B150">
-        <v>2832.3647338745873</v>
+        <v>2466.6232932775529</v>
       </c>
     </row>
     <row r="151" spans="1:2" x14ac:dyDescent="0.3">
@@ -1936,7 +3042,7 @@
         <v>3.5302708124244002E-7</v>
       </c>
       <c r="B151">
-        <v>2999.3281347001866</v>
+        <v>2692.0202027467417</v>
       </c>
     </row>
     <row r="152" spans="1:2" x14ac:dyDescent="0.3">
@@ -1944,7 +3050,7 @@
         <v>3.304988723182471E-7</v>
       </c>
       <c r="B152">
-        <v>3173.2122561306778</v>
+        <v>2934.1308818572829</v>
       </c>
     </row>
     <row r="153" spans="1:2" x14ac:dyDescent="0.3">
@@ -1952,7 +3058,7 @@
         <v>3.0940828711554815E-7</v>
       </c>
       <c r="B153">
-        <v>3349.9862027785484</v>
+        <v>3188.0268935044855</v>
       </c>
     </row>
     <row r="154" spans="1:2" x14ac:dyDescent="0.3">
@@ -1960,7 +3066,7 @@
         <v>2.8966358508138864E-7</v>
       </c>
       <c r="B154">
-        <v>3525.2528641364597</v>
+        <v>3448.2235880745829</v>
       </c>
     </row>
     <row r="155" spans="1:2" x14ac:dyDescent="0.3">
@@ -1968,7 +3074,7 @@
         <v>2.7117887927428619E-7</v>
       </c>
       <c r="B155">
-        <v>3694.3086328503778</v>
+        <v>3708.6830397223061</v>
       </c>
     </row>
     <row r="156" spans="1:2" x14ac:dyDescent="0.3">
@@ -1976,7 +3082,7 @@
         <v>2.5387376335337963E-7</v>
       </c>
       <c r="B156">
-        <v>3852.2034281948581</v>
+        <v>3962.800861192065</v>
       </c>
     </row>
     <row r="157" spans="1:2" x14ac:dyDescent="0.3">
@@ -1984,7 +3090,7 @@
         <v>2.3767296328021569E-7</v>
       </c>
       <c r="B157">
-        <v>3993.8004840568315</v>
+        <v>4203.3789192175163</v>
       </c>
     </row>
     <row r="158" spans="1:2" x14ac:dyDescent="0.3">
@@ -1992,7 +3098,7 @@
         <v>2.2250600730000779E-7</v>
       </c>
       <c r="B158">
-        <v>4113.8335807682915</v>
+        <v>4422.5856820084582</v>
       </c>
     </row>
     <row r="159" spans="1:2" x14ac:dyDescent="0.3">
@@ -2000,7 +3106,7 @@
         <v>2.0830692135334767E-7</v>
       </c>
       <c r="B159">
-        <v>4206.9605973831467</v>
+        <v>4611.9081557745703</v>
       </c>
     </row>
     <row r="160" spans="1:2" x14ac:dyDescent="0.3">
@@ -2008,7 +3114,7 @@
         <v>1.950139414731742E-7</v>
       </c>
       <c r="B160">
-        <v>4267.813199207927</v>
+        <v>4762.1013708116379</v>
       </c>
     </row>
     <row r="161" spans="1:2" x14ac:dyDescent="0.3">
@@ -2016,7 +3122,7 @@
         <v>1.8256924522763054E-7</v>
       </c>
       <c r="B161">
-        <v>4291.0414318698922</v>
+        <v>4863.1407516208174</v>
       </c>
     </row>
     <row r="162" spans="1:2" x14ac:dyDescent="0.3">
@@ -2024,7 +3130,7 @@
         <v>1.7091869947130074E-7</v>
       </c>
       <c r="B162">
-        <v>4271.3527168743676</v>
+        <v>4904.1835975594831</v>
       </c>
     </row>
     <row r="163" spans="1:2" x14ac:dyDescent="0.3">
@@ -2032,7 +3138,7 @@
         <v>1.6001162629770975E-7</v>
       </c>
       <c r="B163">
-        <v>4203.5457455910946</v>
+        <v>4873.5468087695735</v>
       </c>
     </row>
     <row r="164" spans="1:2" x14ac:dyDescent="0.3">
@@ -2040,7 +3146,7 @@
         <v>1.4980058137376085E-7</v>
       </c>
       <c r="B164">
-        <v>4082.5391466213273</v>
+        <v>4758.7068298248478</v>
       </c>
     </row>
     <row r="165" spans="1:2" x14ac:dyDescent="0.3">
@@ -2048,7 +3154,7 @@
         <v>1.4024114815002941E-7</v>
       </c>
       <c r="B165">
-        <v>3903.3948806591743</v>
+        <v>4546.3269460466645</v>
       </c>
     </row>
     <row r="166" spans="1:2" x14ac:dyDescent="0.3">
@@ -2056,7 +3162,7 @@
         <v>1.3129174433611091E-7</v>
       </c>
       <c r="B166">
-        <v>3661.3372399981572</v>
+        <v>4222.3171027190192</v>
       </c>
     </row>
     <row r="167" spans="1:2" x14ac:dyDescent="0.3">
@@ -2064,7 +3170,7 @@
         <v>1.2291344161497093E-7</v>
       </c>
       <c r="B167">
-        <v>3351.7682914364314</v>
+        <v>3771.9301170945273</v>
       </c>
     </row>
     <row r="168" spans="1:2" x14ac:dyDescent="0.3">
@@ -2072,7 +3178,7 @@
         <v>1.1506979461593862E-7</v>
       </c>
       <c r="B168">
-        <v>2970.2790630332711</v>
+        <v>3179.8949866860535</v>
       </c>
     </row>
     <row r="169" spans="1:2" x14ac:dyDescent="0.3">
@@ -2080,7 +3186,7 @@
         <v>1.0772668555528387E-7</v>
       </c>
       <c r="B169">
-        <v>2512.6594922107279</v>
+        <v>2430.5910470007507</v>
       </c>
     </row>
     <row r="170" spans="1:2" x14ac:dyDescent="0.3">
@@ -2088,7 +3194,7 @@
         <v>1.0085217222773789E-7</v>
       </c>
       <c r="B170">
-        <v>1974.9056609371464</v>
+        <v>1508.2598752763795</v>
       </c>
     </row>
     <row r="171" spans="1:2" x14ac:dyDescent="0.3">
@@ -2096,7 +3202,7 @@
         <v>9.4416352428013196E-8</v>
       </c>
       <c r="B171">
-        <v>1353.2265227172259</v>
+        <v>397.25524728801531</v>
       </c>
     </row>
     <row r="172" spans="1:2" x14ac:dyDescent="0.3">
@@ -2104,7 +3210,7 @@
         <v>8.8391230267184831E-8</v>
       </c>
       <c r="B172">
-        <v>644.04950735481998</v>
+        <v>0</v>
       </c>
     </row>
     <row r="173" spans="1:2" x14ac:dyDescent="0.3">
@@ -2321,6 +3427,50 @@
       </c>
       <c r="B199">
         <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0DF158AE-E402-4797-8812-23AC455833B1}">
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B2">
+        <v>0.11559777604404353</v>
+      </c>
+      <c r="C2">
+        <v>0.10765628716758475</v>
+      </c>
+      <c r="D2">
+        <v>8.6506854562582003</v>
+      </c>
+      <c r="E2">
+        <v>9.2888211762619601</v>
       </c>
     </row>
   </sheetData>

</xml_diff>